<commit_message>
breakdown docs and testing
work on backend of new breakdown deliverable
</commit_message>
<xml_diff>
--- a/results/10-2025/beta/inputs-10-2025.xlsx
+++ b/results/10-2025/beta/inputs-10-2025.xlsx
@@ -2183,7 +2183,7 @@
         <v>3310.58125327749</v>
       </c>
       <c r="Q11" t="n">
-        <v>4683.28141700098</v>
+        <v>4936.98141700098</v>
       </c>
       <c r="R11" t="n">
         <v>2509.69750395893</v>
@@ -2240,7 +2240,7 @@
         <v>333.393574536235</v>
       </c>
       <c r="AJ11" t="n">
-        <v>-2773.98977004012</v>
+        <v>-2804.43377004012</v>
       </c>
       <c r="AK11" t="n">
         <v>-1457.24370047507</v>
@@ -2341,7 +2341,7 @@
         <v>3341.68181349335</v>
       </c>
       <c r="Q12" t="n">
-        <v>4711.24089286239</v>
+        <v>5021.94089286239</v>
       </c>
       <c r="R12" t="n">
         <v>2535.4148309503</v>
@@ -2392,13 +2392,13 @@
         <v>0</v>
       </c>
       <c r="AH12" t="n">
-        <v>1952.97849763588</v>
+        <v>1952.94821970685</v>
       </c>
       <c r="AI12" t="n">
-        <v>336.606986627065</v>
+        <v>336.592264556095</v>
       </c>
       <c r="AJ12" t="n">
-        <v>-2784.53667718361</v>
+        <v>-2852.26467718361</v>
       </c>
       <c r="AK12" t="n">
         <v>-1473.99748018911</v>
@@ -2443,10 +2443,10 @@
         <v>0.250425</v>
       </c>
       <c r="AY12" t="n">
-        <v>1700.78675759301</v>
+        <v>1700.77994505898</v>
       </c>
       <c r="AZ12" t="n">
-        <v>293.761926261743</v>
+        <v>293.758613795774</v>
       </c>
     </row>
     <row r="13">
@@ -2499,7 +2499,7 @@
         <v>3373.66737243847</v>
       </c>
       <c r="Q13" t="n">
-        <v>4719.33388949894</v>
+        <v>5030.93734741117</v>
       </c>
       <c r="R13" t="n">
         <v>2559.05905860302</v>
@@ -2550,13 +2550,13 @@
         <v>0</v>
       </c>
       <c r="AH13" t="n">
-        <v>1988.42126832392</v>
+        <v>1988.39059212442</v>
       </c>
       <c r="AI13" t="n">
-        <v>341.03338782625</v>
+        <v>341.018472159202</v>
       </c>
       <c r="AJ13" t="n">
-        <v>-2806.40585890342</v>
+        <v>-2896.30427385289</v>
       </c>
       <c r="AK13" t="n">
         <v>-1490.97271698393</v>
@@ -2601,10 +2601,10 @@
         <v>0.222075</v>
       </c>
       <c r="AY13" t="n">
-        <v>1740.63184296589</v>
+        <v>1740.61812828697</v>
       </c>
       <c r="AZ13" t="n">
-        <v>299.289138522649</v>
+        <v>299.282470031595</v>
       </c>
     </row>
     <row r="14">
@@ -2657,7 +2657,7 @@
         <v>3403.4892424388</v>
       </c>
       <c r="Q14" t="n">
-        <v>4759.66728605607</v>
+        <v>5072.21076771607</v>
       </c>
       <c r="R14" t="n">
         <v>2583.69345621437</v>
@@ -2708,13 +2708,13 @@
         <v>0</v>
       </c>
       <c r="AH14" t="n">
-        <v>2025.63003733759</v>
+        <v>2025.59890969204</v>
       </c>
       <c r="AI14" t="n">
-        <v>344.421964455726</v>
+        <v>344.406900583597</v>
       </c>
       <c r="AJ14" t="n">
-        <v>-2827.4954796584</v>
+        <v>-2936.25711240707</v>
       </c>
       <c r="AK14" t="n">
         <v>-1507.07504187264</v>
@@ -2759,10 +2759,10 @@
         <v>0.1953</v>
       </c>
       <c r="AY14" t="n">
-        <v>1773.92510136685</v>
+        <v>1773.90438296768</v>
       </c>
       <c r="AZ14" t="n">
-        <v>304.977580525187</v>
+        <v>304.967522662904</v>
       </c>
     </row>
     <row r="15">
@@ -2815,7 +2815,7 @@
         <v>3433.8730194392</v>
       </c>
       <c r="Q15" t="n">
-        <v>4800.35923327239</v>
+        <v>5113.879647048</v>
       </c>
       <c r="R15" t="n">
         <v>2606.14312342119</v>
@@ -2866,13 +2866,13 @@
         <v>0</v>
       </c>
       <c r="AH15" t="n">
-        <v>2061.30465790122</v>
+        <v>2061.27317047419</v>
       </c>
       <c r="AI15" t="n">
-        <v>350.086697956147</v>
+        <v>350.0713863274</v>
       </c>
       <c r="AJ15" t="n">
-        <v>-2848.77655428115</v>
+        <v>-2976.46442920816</v>
       </c>
       <c r="AK15" t="n">
         <v>-1522.262673167</v>
@@ -2917,10 +2917,10 @@
         <v>0.171675</v>
       </c>
       <c r="AY15" t="n">
-        <v>1806.37525376969</v>
+        <v>1806.34745069944</v>
       </c>
       <c r="AZ15" t="n">
-        <v>308.733533294667</v>
+        <v>308.720030315916</v>
       </c>
     </row>
     <row r="16">
@@ -2973,7 +2973,7 @@
         <v>3463.52454615578</v>
       </c>
       <c r="Q16" t="n">
-        <v>4841.41363697901</v>
+        <v>5155.94823697901</v>
       </c>
       <c r="R16" t="n">
         <v>2630.50103083491</v>
@@ -3024,13 +3024,13 @@
         <v>0</v>
       </c>
       <c r="AH16" t="n">
-        <v>2080.30849834676</v>
+        <v>2080.27652213188</v>
       </c>
       <c r="AI16" t="n">
-        <v>349.04455464834</v>
+        <v>349.029024808361</v>
       </c>
       <c r="AJ16" t="n">
-        <v>-2868.74815355527</v>
+        <v>-3015.42757158268</v>
       </c>
       <c r="AK16" t="n">
         <v>-1536.70518949433</v>
@@ -3075,10 +3075,10 @@
         <v>0.14805</v>
       </c>
       <c r="AY16" t="n">
-        <v>1835.02450392963</v>
+        <v>1834.99631874507</v>
       </c>
       <c r="AZ16" t="n">
-        <v>311.531986099454</v>
+        <v>311.518301372676</v>
       </c>
     </row>
     <row r="17">
@@ -3131,7 +3131,7 @@
         <v>3492.52886324142</v>
       </c>
       <c r="Q17" t="n">
-        <v>4988.68956051451</v>
+        <v>5304.27594982741</v>
       </c>
       <c r="R17" t="n">
         <v>2656.2474587717</v>
@@ -3182,13 +3182,13 @@
         <v>0</v>
       </c>
       <c r="AH17" t="n">
-        <v>2111.78726525269</v>
+        <v>2111.75480289732</v>
       </c>
       <c r="AI17" t="n">
-        <v>354.248570478128</v>
+        <v>354.232809098846</v>
       </c>
       <c r="AJ17" t="n">
-        <v>-2896.71534682067</v>
+        <v>-3062.45390673909</v>
       </c>
       <c r="AK17" t="n">
         <v>-1551.48029714166</v>
@@ -3233,10 +3233,10 @@
         <v>0.124425</v>
       </c>
       <c r="AY17" t="n">
-        <v>1862.78185323861</v>
+        <v>1862.75326616897</v>
       </c>
       <c r="AZ17" t="n">
-        <v>314.505402196127</v>
+        <v>314.491527184096</v>
       </c>
     </row>
     <row r="18">
@@ -3289,7 +3289,7 @@
         <v>3522.3379634022</v>
       </c>
       <c r="Q18" t="n">
-        <v>5020.29419617941</v>
+        <v>5336.9703301425</v>
       </c>
       <c r="R18" t="n">
         <v>2679.99102251719</v>
@@ -3340,13 +3340,13 @@
         <v>0</v>
       </c>
       <c r="AH18" t="n">
-        <v>2143.75965743293</v>
+        <v>2143.72670077691</v>
       </c>
       <c r="AI18" t="n">
-        <v>359.512864384407</v>
+        <v>359.496868783904</v>
       </c>
       <c r="AJ18" t="n">
-        <v>-2911.99583214346</v>
+        <v>-3096.86345213745</v>
       </c>
       <c r="AK18" t="n">
         <v>-1565.81915799363</v>
@@ -3391,10 +3391,10 @@
         <v>0.1008</v>
       </c>
       <c r="AY18" t="n">
-        <v>1889.36101776006</v>
+        <v>1889.33201916307</v>
       </c>
       <c r="AZ18" t="n">
-        <v>317.90085468008</v>
+        <v>317.886770029165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>